<commit_message>
added special marks from clients
</commit_message>
<xml_diff>
--- a/input_files/Gold_bond.xlsx
+++ b/input_files/Gold_bond.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alon\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2fcf9ad746f2b86b/מסמכים/dormeco-sorting-script/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{6AA09445-608D-47D6-BA55-2C3F9085A174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4E29C120-2BB6-411F-A457-1D6601F21BC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4E29C120-2BB6-411F-A457-1D6601F21BC6}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -135,9 +135,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא של Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -175,7 +175,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -281,7 +281,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -423,7 +423,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -432,14 +432,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F34CDD4-7AD3-4AFF-A586-43E9AE70B2DF}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -450,7 +450,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,7 +461,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,7 +483,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,7 +494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,7 +505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -516,7 +516,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
@@ -527,7 +527,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +538,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>